<commit_message>
Site Plan excel update
</commit_message>
<xml_diff>
--- a/client/Site Plan.xlsx
+++ b/client/Site Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UoB\Research Methodologies\Project\Project\client\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB228201-B7B3-425C-B2C3-CED38B585906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8C2834-ABB5-4DD9-8EB2-9D867C760D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
   <si>
     <t>Internal/ External</t>
   </si>
   <si>
-    <t xml:space="preserve">Role Description </t>
-  </si>
-  <si>
     <t>Access given to that role</t>
   </si>
   <si>
@@ -45,39 +42,6 @@
     <t>Internal</t>
   </si>
   <si>
-    <t>Master Role, Administrator</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Full access
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Special-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Delete projects
-Delete users
-Change User profile settings on users requests</t>
-    </r>
-  </si>
-  <si>
     <t>Director</t>
   </si>
   <si>
@@ -147,10 +111,197 @@
     <t>Manager</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Budget Form access denied
+    <t>Budget Form access denied
+Delete project Confimation access denied (confirmation denied)
+User project deletion access denied (confimation denied)</t>
+  </si>
+  <si>
+    <t>Budget Form access denied
 Delete project Confimation access denied (confirmation denied)
 User project deletion access denied (confimation denied)
+User mgt denied access</t>
+  </si>
+  <si>
+    <t>Denied Access</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Personalized budget view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial user view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Expendtiure access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Updates access (finance)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Full Modal bank access
+Full Location bank access
+View Contact book access</t>
+    </r>
+  </si>
+  <si>
+    <t>Budget Form access denied
+Delete project Confimation access denied (confirmation denied)
+User project deletion access denied (confimation denied)
+User mgt denied access
+User verification level denied
+Full Account access denied
+Denied document creation access</t>
+  </si>
+  <si>
+    <t>Budget Form access denied
+Delete project Confimation access denied
+User project deletion access denied
+User mgt denied access
+User verification level denied
+Full Account access denied</t>
+  </si>
+  <si>
+    <t>Budget Form access denied
+Delete project Confimation access denied
+User project deletion access denied
+User mgt denied access
+User verification level denied</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Full access
 </t>
     </r>
     <r>
@@ -162,38 +313,641 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Special-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-User verification level assign
-Full budget view access
-Full schedule view access
+      <t xml:space="preserve">Special-
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Budget form access
+Delete projects confimation access
+Delete users confimation access
+Change User profile settings on users requests</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Full budget Entry access
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>finance document creation access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial user view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Full Expendtiure access
+Full Accounts access
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Updates access (finance)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Full Modal bank access
+Full Location bank access
+View Contact book access</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Full budget Entry view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial document creation access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial user view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Expendtiure access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Updates access (finance)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Full Modal bank access
+Full Location bank access
+View Contact book access</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">User verification level assign
+Full budget Entry access
+Full schedule access
 Ful document creation access
 Full project detail access
-Full user view access / user mgt partial access
+Full user view access
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>User mgt partial access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
 Full Expendtiure access
 Full Accounts access
 Full Updates access
 Full Hierachy access
 Full Modal bank access
 Full Location bank access
-Full Contanct book access</t>
-    </r>
+Full Contact book access</t>
+    </r>
+  </si>
+  <si>
+    <t>User verification level assign
+Full budget Entry access
+Full schedule access
+Ful document creation access
+Full project detail access
+Full user view access
+Full Expendtiure access
+Full Accounts access
+Full Updates access
+Full Hierachy access
+Full Modal bank access
+Full Location bank access
+Full Contact book access</t>
+  </si>
+  <si>
+    <t>Department Head</t>
+  </si>
+  <si>
+    <t>5 +</t>
+  </si>
+  <si>
+    <t>changeable</t>
+  </si>
+  <si>
+    <t>External</t>
+  </si>
+  <si>
+    <t>Crew</t>
+  </si>
+  <si>
+    <t>20 +</t>
+  </si>
+  <si>
+    <t>Techincial Advisor / Art Director / Gaffer (changeable</t>
+  </si>
+  <si>
+    <t>(changeable)</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Personalized budget view access
+Partial Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail partial view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Updates view access (project)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Personalized budget view access
+Department Budget view access
+Department crew list editing access
+Equipment editing acccess</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail partial view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Expendtiure access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Updates access (project)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access</t>
+    </r>
+  </si>
+  <si>
+    <t>Budget Form access denied
+Delete project Confimation access denied (confirmation denied)
+User project deletion access denied (confimation denied)
+User mgt denied access
+User verification level denied
+Full Account access denied
+Denied document creation access
+Denied user view access
+Denied Modal bank access
+Denied Location bank access
+Denied Contact book access
+Denied Department crew list editing access
+Denied Equipment editing acccess
+Denied Expendtiure access</t>
+  </si>
+  <si>
+    <t>Budget Form access denied
+Delete project Confimation access denied (confirmation denied)
+User project deletion access denied (confimation denied)
+User mgt denied access
+User verification level denied
+Full Account access denied
+Denied document creation access
+Denied user view access
+Denied Modal bank access
+Denied Location bank access
+Denied Contact book access</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -213,6 +967,19 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -238,12 +1005,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -252,16 +1016,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -285,6 +1053,9 @@
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -301,17 +1072,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}" name="Table2" displayName="Table2" ref="A2:H8" totalsRowShown="0" headerRowDxfId="9" dataDxfId="0">
-  <autoFilter ref="A2:H8" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}" name="Table2" displayName="Table2" ref="A2:H16" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A2:H16" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}"/>
   <tableColumns count="8">
-    <tableColumn id="2" xr3:uid="{2E7F7124-D54E-4B29-9BAA-1E6280464E53}" name="Site Role" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{4B71E320-7583-4CD1-AAAD-262148F9FBE6}" name="No of Persons" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{25DEA520-4D59-4E28-81D3-14ECA89E4D3F}" name="VDV Adminsitration Role" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{CAE2965F-B5FB-49E8-B3FC-AC15358FA6F7}" name="Project Role" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{ED20C62D-58EC-43B7-843D-C084ECF6CECD}" name="Verfied Level" dataDxfId="4"/>
-    <tableColumn id="1" xr3:uid="{8DC55ECD-2F56-417D-A5C4-7D97F4E92289}" name="Internal/ External" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{7FDB93E0-60A3-4101-952A-B0D22E3AEAC5}" name="Role Description " dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{2E7F7124-D54E-4B29-9BAA-1E6280464E53}" name="Site Role" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{4B71E320-7583-4CD1-AAAD-262148F9FBE6}" name="No of Persons" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{25DEA520-4D59-4E28-81D3-14ECA89E4D3F}" name="VDV Adminsitration Role" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{CAE2965F-B5FB-49E8-B3FC-AC15358FA6F7}" name="Project Role" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{ED20C62D-58EC-43B7-843D-C084ECF6CECD}" name="Verfied Level" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{8DC55ECD-2F56-417D-A5C4-7D97F4E92289}" name="Internal/ External" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{D8FE2823-BB86-4FF3-91A3-CC7001C345B9}" name="Access given to that role" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{4108AE1A-F3CF-46F7-91AD-435B6F48F159}" name="Denied Access" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -580,46 +1351,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="63.85546875" customWidth="1"/>
+    <col min="7" max="7" width="63.85546875" customWidth="1"/>
+    <col min="8" max="8" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+    <row r="1" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
-    <row r="2" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>0</v>
@@ -628,150 +1398,279 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2">
         <v>2</v>
       </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="5" spans="1:11" ht="195" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="2">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3">
+      <c r="G5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="2">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>7</v>
+      <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="255" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="3">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="3" t="s">
+    <row r="7" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="4" t="s">
+      <c r="F7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>31</v>
       </c>
+      <c r="H8" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="3">
-        <v>2</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="3">
-        <v>1</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+    <row r="10" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="3">
-        <v>1</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+    <row r="11" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
RBAC Site plan updated
</commit_message>
<xml_diff>
--- a/client/Site Plan.xlsx
+++ b/client/Site Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UoB\Research Methodologies\Project\Project\client\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8C2834-ABB5-4DD9-8EB2-9D867C760D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70BF68B4-4D29-4C33-A373-4D61EC2BC392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="60">
   <si>
     <t>Internal/ External</t>
   </si>
@@ -123,157 +123,6 @@
   </si>
   <si>
     <t>Denied Access</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Personalized budget view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Schedule view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Project detail view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Partial user view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Partial Expendtiure access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Partial Updates access (finance)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Hierachy view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Full Modal bank access
-Full Location bank access
-View Contact book access</t>
-    </r>
   </si>
   <si>
     <t>Budget Form access denied
@@ -419,178 +268,6 @@
       <t xml:space="preserve">
 Full Expendtiure access
 Full Accounts access
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Partial Updates access (finance)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Hierachy view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Full Modal bank access
-Full Location bank access
-View Contact book access</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Full budget Entry view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Schedule view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Partial document creation access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Project detail view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Partial user view access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Partial Expendtiure access</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
 </t>
     </r>
     <r>
@@ -924,10 +601,94 @@
 Denied user view access
 Denied Modal bank access
 Denied Location bank access
-Denied Contact book access
-Denied Department crew list editing access
-Denied Equipment editing acccess
-Denied Expendtiure access</t>
+Denied Contact book access</t>
+  </si>
+  <si>
+    <t>Gold level 1</t>
+  </si>
+  <si>
+    <t>Artist
+Producer
+Director
+Corporate client
+Colloborated production house</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Full budget view access (profits hidden)
+Full Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail ful view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Updates view access (project)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access
+Partial Project Blog editor access</t>
+    </r>
   </si>
   <si>
     <t>Budget Form access denied
@@ -937,10 +698,425 @@
 User verification level denied
 Full Account access denied
 Denied document creation access
-Denied user view access
 Denied Modal bank access
 Denied Location bank access
-Denied Contact book access</t>
+Denied Contact book access
+Denied Department crew list editing access
+Denied Equipment editing acccess
+Denied Expendtiure access</t>
+  </si>
+  <si>
+    <t>Client (full access)</t>
+  </si>
+  <si>
+    <t>Client (half access)</t>
+  </si>
+  <si>
+    <t>Cast
+Actor / Actress
+Modal
+Child Actor
+Extras</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Personalized budget view access (profits hidden)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial user view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Expendtiure access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Updates access (finance)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Full Modal bank access
+Full Location bank access
+View Contact book access</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Full budget Entry view access (profits hidden)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial document creation access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial user view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Expendtiure access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partial Updates access (finance)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Full Modal bank access
+Full Location bank access
+View Contact book access</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>personalized budget view access (profits hidden)
+Full Schedule view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Project detail partial view access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Updates view access (project)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hierachy view access
+Partial Project Blog editor access</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1005,7 +1181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1019,10 +1195,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1072,8 +1244,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}" name="Table2" displayName="Table2" ref="A2:H16" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A2:H16" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}" name="Table2" displayName="Table2" ref="A2:H14" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A2:H14" xr:uid="{EA3C247A-1A35-4A96-852B-698FC1A18457}"/>
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{2E7F7124-D54E-4B29-9BAA-1E6280464E53}" name="Site Role" dataDxfId="7"/>
     <tableColumn id="8" xr3:uid="{4B71E320-7583-4CD1-AAAD-262148F9FBE6}" name="No of Persons" dataDxfId="6"/>
@@ -1351,10 +1523,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.5703125" bestFit="1" customWidth="1"/>
@@ -1364,7 +1536,7 @@
     <col min="8" max="8" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -1375,7 +1547,7 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="2" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1401,7 +1573,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1421,11 +1593,11 @@
         <v>4</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="210" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -1444,15 +1616,14 @@
       <c r="F4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="5" t="s">
+      <c r="G4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="195" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="195" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -1472,13 +1643,13 @@
         <v>4</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="180" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -1498,13 +1669,13 @@
         <v>4</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1524,13 +1695,13 @@
         <v>4</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -1550,13 +1721,13 @@
         <v>4</v>
       </c>
       <c r="G8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>32</v>
-      </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1566,59 +1737,59 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="D10" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="195" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>52</v>
+      <c r="C11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="210" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1628,45 +1799,57 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+    <row r="13" spans="1:8" ht="195" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+    <row r="14" spans="1:8" ht="195" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>